<commit_message>
[UPDATE]: Complete project documentation
</commit_message>
<xml_diff>
--- a/documentation/Sprint Backlog Burndown.xlsx
+++ b/documentation/Sprint Backlog Burndown.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Related User Story</t>
   </si>
@@ -95,9 +95,6 @@
   </si>
   <si>
     <t>Perform manual testing and update documentation</t>
-  </si>
-  <si>
-    <t>Tests unitaires à chaque implémentations</t>
   </si>
   <si>
     <t>Estimate Totals</t>
@@ -132,7 +129,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -167,12 +164,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE599"/>
-        <bgColor rgb="FFFFE599"/>
       </patternFill>
     </fill>
     <fill>
@@ -218,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -237,18 +228,27 @@
     <xf borderId="6" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="6" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="6" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
     <xf borderId="6" fillId="5" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="6" fillId="6" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="6" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="6" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="6" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="6" fillId="8" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="6" fillId="8" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="6" fillId="7" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -313,11 +313,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="922454891"/>
-        <c:axId val="1480661311"/>
+        <c:axId val="1110647532"/>
+        <c:axId val="1334329534"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="922454891"/>
+        <c:axId val="1110647532"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -373,10 +373,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1480661311"/>
+        <c:crossAx val="1334329534"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1480661311"/>
+        <c:axId val="1334329534"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -442,7 +442,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="922454891"/>
+        <c:crossAx val="1110647532"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -736,10 +736,18 @@
       <c r="C3" s="9">
         <v>1.5</v>
       </c>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
+      <c r="D3" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E3" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G3" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8"/>
@@ -749,10 +757,18 @@
       <c r="C4" s="9">
         <v>2.0</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
+      <c r="D4" s="10">
+        <v>2.0</v>
+      </c>
+      <c r="E4" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G4" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
@@ -764,10 +780,18 @@
       <c r="C5" s="9">
         <v>1.5</v>
       </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
+      <c r="D5" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E5" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="F5" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G5" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8"/>
@@ -777,10 +801,18 @@
       <c r="C6" s="9">
         <v>0.5</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
+      <c r="D6" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="E6" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G6" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8"/>
@@ -790,10 +822,18 @@
       <c r="C7" s="8">
         <v>1.0</v>
       </c>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+      <c r="D7" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="E7" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G7" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8"/>
@@ -803,10 +843,18 @@
       <c r="C8" s="9">
         <v>2.0</v>
       </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
+      <c r="D8" s="10">
+        <v>2.0</v>
+      </c>
+      <c r="E8" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="F8" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G8" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8"/>
@@ -816,10 +864,18 @@
       <c r="C9" s="8">
         <v>0.5</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
+      <c r="D9" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="G9" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="s">
@@ -831,10 +887,18 @@
       <c r="C10" s="8">
         <v>0.5</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+      <c r="D10" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="F10" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8"/>
@@ -844,10 +908,18 @@
       <c r="C11" s="9">
         <v>1.5</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
+      <c r="D11" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="F11" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="s">
@@ -859,10 +931,18 @@
       <c r="C12" s="8">
         <v>0.5</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
+      <c r="D12" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="F12" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="G12" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8"/>
@@ -872,10 +952,18 @@
       <c r="C13" s="9">
         <v>1.5</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
+      <c r="D13" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E13" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="F13" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="G13" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
@@ -887,10 +975,18 @@
       <c r="C14" s="8">
         <v>0.5</v>
       </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
+      <c r="D14" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="G14" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8"/>
@@ -900,179 +996,201 @@
       <c r="C15" s="9">
         <v>1.5</v>
       </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
+      <c r="D15" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E15" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="F15" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="G15" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="15">
         <v>1.5</v>
       </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="D16" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E16" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F16" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="G16" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8"/>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="15">
         <v>1.0</v>
       </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="D17" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="E17" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="F17" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="G17" s="16">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
     </row>
     <row r="19">
       <c r="A19" s="8"/>
-      <c r="B19" s="13" t="s">
-        <v>28</v>
-      </c>
+      <c r="B19" s="8"/>
       <c r="C19" s="8"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
     </row>
     <row r="20">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="B31" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C31" s="15">
+      <c r="B31" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="18">
         <f t="shared" ref="C31:G31" si="1">SUM(C3:C30)</f>
         <v>17.5</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="18">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E31" s="15">
+        <v>17.5</v>
+      </c>
+      <c r="E31" s="18">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F31" s="15">
+        <v>11</v>
+      </c>
+      <c r="F31" s="18">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G31" s="15">
+        <v>6</v>
+      </c>
+      <c r="G31" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>

</xml_diff>